<commit_message>
sch+pcb: eurorack I/O stage — input pad 100k/39k, TL072 x4.9 output amp on ±12V
- input divider now populated (R2/R3 = 100k/39k, -11.5dB): ±5V modular
  swings land inside the hat codec range; also protects against CV/gate
  mis-patches. Guitar-level alternative (R2=0R, R3 off) documented
- output: TL072 (C6961) x4.9 on +12V_F and a newly conditioned -12V rail
  (D2 SS34 + FB2 bead + 100n/22u), hat ~2Vpp -> ~10Vpp modular level,
  1k series out; spare half terminated; AOUT_S bonded to GND at one
  point (NT1 net tie); PWR_FLAG on -12V_F
- all new parts placed + routed, DRC clean; audit: no aggressors near
  the input pair, amp output >=3mm from input path everywhere
- fp-lib-table: add Package_SO + NetTie; BOM: 3 new lines (all LCSC
  in-stock verified), R2/R7 and R3/R5 share parts; ~45c/board added
- fab regen (CPL 19 placements, no DNP); verify D1/D2/U2 rotations in
  JLC preview; doc PDFs + STEP regenerated
</commit_message>
<xml_diff>
--- a/fab/eurorack-BOM.xlsx
+++ b/fab/eurorack-BOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D1, D2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -468,7 +468,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>C1, C3</t>
+          <t>C1, C3, C7</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -490,7 +490,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C2, C4</t>
+          <t>C2, C4, C5, C6</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -512,7 +512,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FB1</t>
+          <t>FB1, FB2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -529,12 +529,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0R jumper</t>
+          <t>100k 1%</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R2, R7</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -544,7 +544,95 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C60485</t>
+          <t>C60491</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>39k 1%</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>R3, R5</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0402</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>C137995</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>10k 1%</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0402</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>C60490</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1k 1%</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0402</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>C106235</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Dual JFET op-amp</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>U2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SOIC-8</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>C6961</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fab: full JLC assembly — THT parts join BOM+CPL (28 placements); J4/J5 now a real 1x7 header (XFCN PZ254V-11-07P, C492406) instead of snap-from-strip
</commit_message>
<xml_diff>
--- a/fab/eurorack-BOM.xlsx
+++ b/fab/eurorack-BOM.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,78 +441,78 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Schottky reverse protection 40V 3A</t>
+          <t>Eurorack power header 2x5 shrouded IDC</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>D1, D2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SMA (DO-214AC)</t>
+          <t>IDC box 2x5 P2.54mm</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>C8678</t>
+          <t>C5665</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>22uF 25V X5R</t>
+          <t>5V/1A buck module (7805 drop-in)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>C1, C3, C7</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>SIP-3 (TSR-1 land, P2.54)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>C398931</t>
+          <t>C2992391</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>100nF 50V X7R</t>
+          <t>Schottky reverse protection 40V 3A</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>C2, C4, C5, C6</t>
+          <t>D1, D2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>SMA (DO-214AC)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C131394</t>
+          <t>C8678</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ferrite bead 600R@100MHz 2A</t>
+          <t>22uF 25V X5R</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FB1, FB2</t>
+          <t>C1, C3, C7</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -522,19 +522,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C21519</t>
+          <t>C398931</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>100k 1%</t>
+          <t>100nF 50V X7R</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>R2, R7</t>
+          <t>C2, C4, C5, C6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -544,41 +544,41 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C60491</t>
+          <t>C131394</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>39k 1%</t>
+          <t>Ferrite bead 600R@100MHz 2A</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>R3, R5</t>
+          <t>FB1, FB2</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>C137995</t>
+          <t>C21519</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10k 1%</t>
+          <t>100k 1%</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R2, R7</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -588,19 +588,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>C60490</t>
+          <t>C60491</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1k 1%</t>
+          <t>39k 1%</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>R6</t>
+          <t>R3, R5</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -610,27 +610,181 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>C106235</t>
+          <t>C137995</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>1x7 female socket 8.5mm stack</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>J2, J3</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PinSocket 1x7 P2.54 TH</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>C2832270</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1x7 male header</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>J4, J5</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PinHeader 1x7 P2.54 TH</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>C492406</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1x4 male header</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>J8</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PinHeader 1x4 P2.54 TH</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>C124378</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3.5mm mono jack, horizontal, threaded</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>J6, J7</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Vertical THT nose-up, M7.7x0.75 plastic thread</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>C5146694</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1x4 female socket, 8.5mm</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>J10</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>PinSocket 1x4 P2.54 TH (H85)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>C541851</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10k 1%</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>0402</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>C60490</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1k 1%</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0402</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>C106235</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>Dual JFET op-amp</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>U2</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>SOIC-8</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>C6961</t>
         </is>

</xml_diff>